<commit_message>
Update TCCC Variable Definitions
</commit_message>
<xml_diff>
--- a/dashboard-ui/src/components/Research/variables/Variable Definitions TCCC.xlsx
+++ b/dashboard-ui/src/components/Research/variables/Variable Definitions TCCC.xlsx
@@ -5,22 +5,22 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gary.cheng_cn\Projects\itm-evaluation-dashboard\dashboard-ui\src\components\Research\variables\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gary.cheng_cn\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F72503F9-BC13-4F47-9A95-63EE6295D9EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{72B709A4-92EF-4A27-A6F8-54CA82AAD129}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{B335D1ED-2780-4984-A298-197D94347E3F}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{C225C15C-1D6D-4CFE-A0FB-ABC62FC30937}"/>
   </bookViews>
   <sheets>
-    <sheet name="tccc_field_definitions" sheetId="1" r:id="rId1"/>
+    <sheet name="Variable Definitions TCCC" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="86">
   <si>
     <t>Field Name</t>
   </si>
@@ -85,9 +85,6 @@
     <t>TCCC Hemorrhage control</t>
   </si>
   <si>
-    <t>TCCC Hemorrhage control_time</t>
-  </si>
-  <si>
     <t>{Patient} Time</t>
   </si>
   <si>
@@ -106,6 +103,9 @@
     <t>{Patient} Tag</t>
   </si>
   <si>
+    <t>1st - {N}th Patient</t>
+  </si>
+  <si>
     <t>{Patient} Time (s)</t>
   </si>
   <si>
@@ -142,10 +142,7 @@
     <t>9-digit participant ID derived from the filename</t>
   </si>
   <si>
-    <t>Elapsed time in seconds from session start until the participant began triaging patients</t>
-  </si>
-  <si>
-    <t>Total number of triage tags applied by the participant across all patients</t>
+    <t>Number of distinct patients the participant tagged (the last tag applied to each patient is the one counted)</t>
   </si>
   <si>
     <t>Proportion of tags that matched the correct triage color for each patient</t>
@@ -160,13 +157,13 @@
     <t>Proportion of tags where participant placed a patient in dead/expectant incorrectly</t>
   </si>
   <si>
-    <t>Percentage score of correct treatments applied out of total tools used plus missed required treatments; (correct tools / (total tools + missed)) * 100</t>
-  </si>
-  <si>
-    <t>Total number of assessment actions performed (SpO2 pulse breathing checks) across all patients</t>
-  </si>
-  <si>
-    <t>Average number of assessment actions performed per patient engaged</t>
+    <t>Total number of combined tagging_errors + missed_hemorrhage + incorrect treatments</t>
+  </si>
+  <si>
+    <t>Number of assessment actions (SpO2/pulse/breathing) across all patients; repeats of the same check type within 5 seconds are not counted again</t>
+  </si>
+  <si>
+    <t>Average number of assessment actions per patient engaged (same-type checks within 5 seconds are de-duplicated)</t>
   </si>
   <si>
     <t>Total number of treatment tools applied across all patients (excluding pulse oximeter)</t>
@@ -175,19 +172,19 @@
     <t>Average number of treatment tools applied per patient treated</t>
   </si>
   <si>
+    <t>Same as Time to Triage Scene; total session duration from session start to the final action before session end</t>
+  </si>
+  <si>
     <t>Average triage time divided by number of patients engaged</t>
   </si>
   <si>
-    <t>Average number of times the participant re-engaged each patient</t>
-  </si>
-  <si>
     <t>Proportion of triage tags that were correct</t>
   </si>
   <si>
     <t>Whether the participant correctly tagged at least one expectant patient as black</t>
   </si>
   <si>
-    <t>Whether the participant performed any hemorrhage control</t>
+    <t>Whether the participant completed all required hemorrhage control (1 only when every required HC procedure is completed)</t>
   </si>
   <si>
     <t>Total time in seconds the participant spent interacting with this specific patient</t>
@@ -196,13 +193,16 @@
     <t>The order in which the participant first engaged this patient</t>
   </si>
   <si>
-    <t>Number of assessment actions performed on this specific patient</t>
+    <t>Whether the participant chose to evacuate this patient</t>
+  </si>
+  <si>
+    <t>Number of assessment actions performed on this specific patient (same-type checks within 5 seconds are de-duplicated)</t>
   </si>
   <si>
     <t>Number of treatment tools applied to this specific patient</t>
   </si>
   <si>
-    <t>Triage tag color the participant assigned to this patient</t>
+    <t>Triage tag color the participant assigned to this patient (raw value; may also appear as yellow_orange / green_blue / gray)</t>
   </si>
   <si>
     <t>Whether the tag applied to the Nth patient in order was correct</t>
@@ -232,7 +232,7 @@
     <t>Integer; 0 to number of patients in scenario</t>
   </si>
   <si>
-    <t>Decimal 0.0 â€“ 1.0</t>
+    <t>Decimal 0.0 - 1.0</t>
   </si>
   <si>
     <t>Integer; 0+</t>
@@ -244,49 +244,40 @@
     <t>Decimal (seconds); 0.0+</t>
   </si>
   <si>
+    <t>Decimal 0.0+</t>
+  </si>
+  <si>
     <t>Yes / No</t>
   </si>
   <si>
     <t>0 (no) / 1 (yes)</t>
   </si>
   <si>
+    <t>Numeric (seconds)</t>
+  </si>
+  <si>
+    <t>Integer 1+</t>
+  </si>
+  <si>
+    <t>red / yellow / green / black (raw values may also include yellow_orange / green_blue / gray)</t>
+  </si>
+  <si>
     <t>0 (incorrect) / 1 (correct)</t>
   </si>
   <si>
     <t>Decimal (seconds)</t>
   </si>
   <si>
-    <t>Decimal 0.0 - 1.0</t>
-  </si>
-  <si>
-    <t>0.0 - 100.0</t>
-  </si>
-  <si>
-    <t>Same as Time to Triage Scene, total time to begin triaging</t>
-  </si>
-  <si>
-    <t>Decimal 0.0+</t>
-  </si>
-  <si>
-    <t>Numeric (seconds)</t>
-  </si>
-  <si>
-    <t>Integer 1+</t>
-  </si>
-  <si>
-    <t>Whether the participant chose to evacuate this patient</t>
-  </si>
-  <si>
-    <t>red / yellow / green / black</t>
-  </si>
-  <si>
-    <t>1st - {N}th Patient</t>
-  </si>
-  <si>
-    <t>Total number of combined tagging_errors + missed_hemorrhage + incorrect treatments</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> time from scene start until all required HC treatments completed; only has a value when flag = 1</t>
+    <t>Percentage score of correct treatments applied out of total tools used plus missed required treatments; (correct tools / (total tools + missed))</t>
+  </si>
+  <si>
+    <t>Elapsed time in seconds from session start  to the final action before session end; i.e. total scene/session duration</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> time from scene start until all required HC treatments completed; only has a value when TCCC Hemorrhage control = 1</t>
+  </si>
+  <si>
+    <t>Average number of engagement visits per patient — the first visit counts as 1 and each return visit adds 1, the value is 1.0 when no patient is revisited and higher when patients are revisited</t>
   </si>
 </sst>
 </file>
@@ -1146,47 +1137,46 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C64312BC-F3F9-4479-ABDB-C040E1EA11E7}">
-  <dimension ref="A1:AH4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9022F6AF-1660-4719-ACB9-EC9BE9EB9D68}">
+  <dimension ref="A1:AG4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.81640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="40.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="75.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="62.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="114.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="91.36328125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="61.90625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="65.1796875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="64.453125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="71.81640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="81.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="75.08984375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="101.7265625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="75.26953125" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="126.54296875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="84.90625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="61.453125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="126.6328125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="100.1796875" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="74.7265625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="53.54296875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="52.453125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="94.453125" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="50.7265625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="56.453125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="161" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="36.36328125" bestFit="1" customWidth="1"/>
     <col min="20" max="20" width="68.54296875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="51.54296875" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="56.54296875" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="68.7265625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="51.36328125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="65.453125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="57.08984375" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="49.90625" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="47.7265625" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="54" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="65.7265625" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="44.453125" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="54.54296875" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="63.26953125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="62.26953125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="106.90625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="68.7265625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="51.36328125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="47" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="105.26953125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="49.90625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="105.08984375" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="54" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="65.7265625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="44.453125" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="54.54296875" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="63.26953125" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="62.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1272,25 +1262,22 @@
         <v>27</v>
       </c>
       <c r="AC1" t="s">
-        <v>86</v>
+        <v>28</v>
       </c>
       <c r="AD1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="AE1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="AF1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="AG1" t="s">
-        <v>31</v>
-      </c>
-      <c r="AH1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="2" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>33</v>
       </c>
@@ -1373,10 +1360,10 @@
         <v>34</v>
       </c>
       <c r="AB2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="AC2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="AD2" t="s">
         <v>36</v>
@@ -1385,16 +1372,13 @@
         <v>36</v>
       </c>
       <c r="AF2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="AG2" t="s">
         <v>37</v>
       </c>
-      <c r="AH2" t="s">
-        <v>37</v>
-      </c>
     </row>
-    <row r="3" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>38</v>
       </c>
@@ -1402,64 +1386,64 @@
         <v>39</v>
       </c>
       <c r="C3" t="s">
+        <v>83</v>
+      </c>
+      <c r="D3" t="s">
         <v>40</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>41</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>42</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>43</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>44</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
+        <v>84</v>
+      </c>
+      <c r="J3" t="s">
         <v>45</v>
       </c>
-      <c r="I3" t="s">
-        <v>88</v>
-      </c>
-      <c r="J3" t="s">
-        <v>87</v>
-      </c>
       <c r="K3" t="s">
+        <v>82</v>
+      </c>
+      <c r="L3" t="s">
         <v>46</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M3" t="s">
         <v>47</v>
       </c>
-      <c r="M3" t="s">
+      <c r="N3" t="s">
         <v>48</v>
       </c>
-      <c r="N3" t="s">
+      <c r="O3" t="s">
         <v>49</v>
       </c>
-      <c r="O3" t="s">
+      <c r="P3" t="s">
         <v>50</v>
-      </c>
-      <c r="P3" t="s">
-        <v>80</v>
       </c>
       <c r="Q3" t="s">
         <v>51</v>
       </c>
       <c r="R3" t="s">
+        <v>85</v>
+      </c>
+      <c r="S3" t="s">
         <v>52</v>
       </c>
-      <c r="S3" t="s">
+      <c r="T3" t="s">
         <v>53</v>
       </c>
-      <c r="T3" t="s">
+      <c r="U3" t="s">
         <v>54</v>
       </c>
-      <c r="U3" t="s">
+      <c r="V3" t="s">
         <v>55</v>
-      </c>
-      <c r="V3" t="s">
-        <v>88</v>
       </c>
       <c r="W3" t="s">
         <v>56</v>
@@ -1468,37 +1452,34 @@
         <v>57</v>
       </c>
       <c r="Y3" t="s">
-        <v>84</v>
+        <v>58</v>
       </c>
       <c r="Z3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="AA3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="AB3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="AC3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="AD3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="AE3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="AF3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="AG3" t="s">
-        <v>65</v>
-      </c>
-      <c r="AH3" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="4" spans="1:34" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:33" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>67</v>
       </c>
@@ -1509,13 +1490,13 @@
         <v>69</v>
       </c>
       <c r="E4" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="F4" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="G4" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="H4" t="s">
         <v>70</v>
@@ -1527,7 +1508,7 @@
         <v>71</v>
       </c>
       <c r="K4" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="L4" t="s">
         <v>71</v>
@@ -1548,55 +1529,52 @@
         <v>73</v>
       </c>
       <c r="R4" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="S4" t="s">
+        <v>70</v>
+      </c>
+      <c r="T4" t="s">
+        <v>75</v>
+      </c>
+      <c r="U4" t="s">
+        <v>76</v>
+      </c>
+      <c r="V4" t="s">
+        <v>77</v>
+      </c>
+      <c r="W4" t="s">
         <v>78</v>
       </c>
-      <c r="T4" t="s">
-        <v>74</v>
-      </c>
-      <c r="U4" t="s">
+      <c r="X4" t="s">
         <v>75</v>
       </c>
-      <c r="V4" t="s">
-        <v>82</v>
-      </c>
-      <c r="W4" t="s">
-        <v>82</v>
-      </c>
-      <c r="X4" t="s">
-        <v>83</v>
-      </c>
       <c r="Y4" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="Z4" t="s">
         <v>71</v>
       </c>
       <c r="AA4" t="s">
+        <v>79</v>
+      </c>
+      <c r="AB4" t="s">
+        <v>80</v>
+      </c>
+      <c r="AC4" t="s">
+        <v>77</v>
+      </c>
+      <c r="AD4" t="s">
         <v>71</v>
       </c>
-      <c r="AB4" t="s">
-        <v>85</v>
-      </c>
-      <c r="AC4" t="s">
-        <v>76</v>
-      </c>
-      <c r="AD4" t="s">
-        <v>82</v>
-      </c>
       <c r="AE4" t="s">
-        <v>71</v>
+        <v>81</v>
       </c>
       <c r="AF4" t="s">
         <v>77</v>
       </c>
       <c r="AG4" t="s">
-        <v>82</v>
-      </c>
-      <c r="AH4" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
TCCC Triage Performance typo
</commit_message>
<xml_diff>
--- a/dashboard-ui/src/components/Research/variables/Variable Definitions TCCC.xlsx
+++ b/dashboard-ui/src/components/Research/variables/Variable Definitions TCCC.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gary.cheng_cn\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{72B709A4-92EF-4A27-A6F8-54CA82AAD129}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{213838A7-30FB-4DC2-B968-06D482EA9101}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{C225C15C-1D6D-4CFE-A0FB-ABC62FC30937}"/>
   </bookViews>
@@ -268,9 +268,6 @@
     <t>Decimal (seconds)</t>
   </si>
   <si>
-    <t>Percentage score of correct treatments applied out of total tools used plus missed required treatments; (correct tools / (total tools + missed))</t>
-  </si>
-  <si>
     <t>Elapsed time in seconds from session start  to the final action before session end; i.e. total scene/session duration</t>
   </si>
   <si>
@@ -278,6 +275,9 @@
   </si>
   <si>
     <t>Average number of engagement visits per patient — the first visit counts as 1 and each return visit adds 1, the value is 1.0 when no patient is revisited and higher when patients are revisited</t>
+  </si>
+  <si>
+    <t>Decimal score of correct treatments applied out of total tools used plus missed required treatments; (correct tools / (total tools + missed))</t>
   </si>
 </sst>
 </file>
@@ -1386,7 +1386,7 @@
         <v>39</v>
       </c>
       <c r="C3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D3" t="s">
         <v>40</v>
@@ -1404,13 +1404,13 @@
         <v>44</v>
       </c>
       <c r="I3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J3" t="s">
         <v>45</v>
       </c>
       <c r="K3" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="L3" t="s">
         <v>46</v>
@@ -1431,7 +1431,7 @@
         <v>51</v>
       </c>
       <c r="R3" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="S3" t="s">
         <v>52</v>

</xml_diff>